<commit_message>
README cleanup; rename "white space" to "open gap"
- Tagline, nav and quick start trimmed; quick start shows the manual
  Claude Code marketplace install. OpenAlex key row removed.
- Ground rules and quadrant meanings rewritten in plain words (EN/ES/CN).
- "White space" is now "open gap" across the README, SKILL.md, engine,
  charts, workbook and example.
- Banner pill removed; gap-matrix illustration explains each quadrant
  in words instead of decorative dots. Gap chart labels get headroom.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0152p1MSwEKBAf7VK4U2fokc
</commit_message>
<xml_diff>
--- a/examples/predictive-maintenance/paradigma_predictive-maintenance.xlsx
+++ b/examples/predictive-maintenance/paradigma_predictive-maintenance.xlsx
@@ -720,7 +720,7 @@
     <row r="5" ht="51" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PARADIGMA asks one question about a field: which of the things that limit it (prices, performance, laws, patents, skills, norms, supply) changed over the chosen years, who is already building on each change, and where something changed but almost nobody is building yet. A limit that fell but nobody uses yet is a possible opening, called white space.</t>
+          <t>PARADIGMA asks one question about a field: which of the things that limit it (prices, performance, laws, patents, skills, norms, supply) changed over the chosen years, who is already building on each change, and where something changed but almost nobody is building yet. A limit that fell but nobody uses yet is a possible opening, called open gap.</t>
         </is>
       </c>
     </row>
@@ -906,19 +906,19 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="21" customHeight="1">
+    <row r="24" ht="36" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>White space</t>
+          <t>Open gap</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Fell a lot, few building. A possible opening, but only after the why-not check.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="21" customHeight="1">
+          <t>The constraint dropped a lot (cheaper, allowed, easier), but few companies use the change yet. A possible opening, but only after the why-not check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Crowded</t>
@@ -926,11 +926,11 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Fell a lot, many already building.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="21" customHeight="1">
+          <t>The constraint dropped a lot and many companies already use it. This is what most people in the field already know.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Hype risk</t>
@@ -938,7 +938,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Little real change, but many building anyway.</t>
+          <t>The constraint barely moved, yet many companies are building on it anyway. A warning sign: lots of activity with no real change underneath.</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Little change and little activity.</t>
+          <t>The constraint barely moved and few are building on it.</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Something else still stands in the way. Goes to a watch list, not to white space.</t>
+          <t>Something else still stands in the way. Goes to a watch list, not to open gap.</t>
         </is>
       </c>
     </row>
@@ -33068,7 +33068,7 @@
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>WHITE SPACE</t>
+          <t>OPEN GAP</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
@@ -33740,7 +33740,7 @@
     <row r="1" ht="21" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Only Untried and Tried too early count as white space. Blocked goes to a watch list.</t>
+          <t>Only Untried and Tried too early count as open gap. Blocked goes to a watch list.</t>
         </is>
       </c>
     </row>

</xml_diff>